<commit_message>
git cleanup and MSAR refresh
</commit_message>
<xml_diff>
--- a/med_school_list_md.xlsx
+++ b/med_school_list_md.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MD Schools'!$A$4:$L$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MD Schools'!$A$4:$L$34</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
     <row r="1" ht="19" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>U.S. MD school list tailored for 3.73 GPA / 514-520 MCAT / California resident / fit-first screening</t>
+          <t>U.S. MD school list refined against live 2027 MSAR data on May 30, 2026</t>
         </is>
       </c>
       <c r="B1" s="10" t="n"/>
@@ -524,7 +524,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>List trimmed away schools with regional-tie or population-specific screens when they looked less likely to improve your real odds; current list favors California, mission fit, and cleaner non-tie lower-tier options.</t>
+          <t>Live MSAR review removed high-stat public/OOS reaches and reclassified several private schools upward in risk; this version is optimized more for realistic odds than prestige coverage.</t>
         </is>
       </c>
       <c r="B2" s="10" t="n"/>
@@ -1543,7 +1543,7 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Kaiser Permanente Bernard J. Tyson School of Medicine</t>
+          <t>Loyola University Chicago Stritch School of Medicine</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1553,17 +1553,17 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Pasadena, CA</t>
+          <t>Maywood, IL</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>39636</v>
+        <v>107024</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>3.87</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
@@ -1587,20 +1587,20 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Strong humanism-and-equity fit; still selective, but more defensible than some of the private prestige schools that were cut.</t>
+          <t>Jesuit social-justice mission fits your community work, though its interview pattern keeps it in target rather than safety territory.</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Kaiser Permanente Bernard J. Tyson School of Medicine strives to provide a world-class education for every one of our students.
-We aim to ignite a passion for lifelong learning, a desire to serve patients, and an unwavering commitment to improve the health and well-being of communities.  </t>
+          <t xml:space="preserve">Loyola University Chicago Stritch School of Medicine (SSOM) is committed to scholarship and the education of medical professionals and biomedical scientists. Our school, including its faculty, trainees, and staff are, called to go beyond facts, experimentation, and treatment of disease to prepare people to lead extraordinary lives and treat the human spirit in an environment that encourages innovation embraces diversity, respects life, and values human dignity.
+</t>
         </is>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Loyola University Chicago Stritch School of Medicine</t>
+          <t>Medical College of Wisconsin</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1610,17 +1610,17 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Maywood, IL</t>
+          <t>Milwaukee, WI</t>
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>107024</v>
+        <v>109187</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>3.87</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
@@ -1644,67 +1644,10 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Jesuit social-justice mission fits your community work, though its interview pattern keeps it in target rather than safety territory.</t>
+          <t>Solid research-plus-service fit with a friendlier statistical profile than the top-heavy schools you cut.</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Loyola University Chicago Stritch School of Medicine (SSOM) is committed to scholarship and the education of medical professionals and biomedical scientists. Our school, including its faculty, trainees, and staff are, called to go beyond facts, experimentation, and treatment of disease to prepare people to lead extraordinary lives and treat the human spirit in an environment that encourages innovation embraces diversity, respects life, and values human dignity.
-</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Medical College of Wisconsin</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Milwaukee, WI</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>109187</v>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>3.87</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>511</v>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>Solid research-plus-service fit with a friendlier statistical profile than the top-heavy schools you cut.</t>
-        </is>
-      </c>
-      <c r="L23" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Our Mission: We are a distinguished leader and innovator in the education and development of the next generation of physicians, scientists, pharmacists and health professionals; we discover and translate new knowledge in the biomedical and health sciences; we provide cutting-edge, collaborative patient care of the highest quality; and we improve the health of the communities we serve.
 Our Vision: Pioneering pathways to a healthier world.
@@ -1713,10 +1656,66 @@
         </is>
       </c>
     </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Nova Southeastern University Dr. Kiran C. Patel College of Allopathic Medicine</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Davie, FL</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>113686</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>513</v>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Added as a cleaner lower-tier replacement because it does not appear to impose the same regional-ties burden as schools like Western Michigan, while still fitting your research, service, and teamwork profile.</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Our mission at NSU MD is advancing human health through innovation in medical education, research, patient care, and community engagement. We will achieve it utilizing a patient-centered, student-centered, and community-centered approach.</t>
+        </is>
+      </c>
+    </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>New York Medical College</t>
+          <t>Sidney Kimmel Medical College at Thomas Jefferson University</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1726,17 +1725,17 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Valhalla, NY</t>
+          <t>Philadelphia, PA</t>
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>102045</v>
+        <v>102480</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>3.89</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
@@ -1760,19 +1759,19 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Private target with room for your high MCAT to help offset GPA risk.</t>
+          <t>Urban clinical environment and broad mission make this a sensible middle-of-list target.</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>New York Medical College is a graduate health sciences university whose purpose is to educate physicians, scientists, public health specialists, and other healthcare professionals, and to conduct biomedical and population-based research. Through its faculty and affiliated clinical partners, the College provides service to its community in an atmosphere of excellence, scholarship, and professionalism. New York Medical College believes the rich diversity of its student body and faculty is important to its mission of educating outstanding health care professionals for the multicultural world of the 21st century. This commitment to diversity and inclusion is woven into the fabric of the institution.  Students come from across the US, representing a broad range of racial, ethnic, cultural, economic, and educational backgrounds.</t>
+          <t xml:space="preserve">Sidney Kimmel Medical College at Thomas Jefferson University is committed to: educating physicians who will form and lead the integrated healthcare delivery and research teams of tomorrow; discovering new knowledge that will define the future of clinical care through investigation from the laboratory to the bedside, and into the community; and setting the standard for quality, compassionate and efficient patient care for our community and for the nation. We recognize that a diverse community is imperative to achieving excellence in patient care, education, and research. As we carry out our mission, we are committed to the highest standards of professionalism and aspire to be a community of discovery, learning, and inclusion. </t>
         </is>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Nova Southeastern University Dr. Kiran C. Patel College of Allopathic Medicine</t>
+          <t>University of Illinois College of Medicine</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1782,17 +1781,17 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Davie, FL</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>113686</v>
+        <v>123095</v>
       </c>
       <c r="E25" s="5" t="n">
         <v>3.85</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -1801,7 +1800,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Public (out-of-state COA)</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -1816,245 +1815,10 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Added as a cleaner lower-tier replacement because it does not appear to impose the same regional-ties burden as schools like Western Michigan, while still fitting your research, service, and teamwork profile.</t>
+          <t>Public-school add with some out-of-state risk, but still a useful lower-tier target because its prompts and mission fit you well and the academic bar is manageable.</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
-        <is>
-          <t>Our mission at NSU MD is advancing human health through innovation in medical education, research, patient care, and community engagement. We will achieve it utilizing a patient-centered, student-centered, and community-centered approach.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Sidney Kimmel Medical College at Thomas Jefferson University</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Philadelphia, PA</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>102480</v>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="F26" s="6" t="n">
-        <v>514</v>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>Urban clinical environment and broad mission make this a sensible middle-of-list target.</t>
-        </is>
-      </c>
-      <c r="L26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sidney Kimmel Medical College at Thomas Jefferson University is committed to: educating physicians who will form and lead the integrated healthcare delivery and research teams of tomorrow; discovering new knowledge that will define the future of clinical care through investigation from the laboratory to the bedside, and into the community; and setting the standard for quality, compassionate and efficient patient care for our community and for the nation. We recognize that a diverse community is imperative to achieving excellence in patient care, education, and research. As we carry out our mission, we are committed to the highest standards of professionalism and aspire to be a community of discovery, learning, and inclusion. </t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>The Ohio State University College of Medicine</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Columbus, OH</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>87056</v>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="F27" s="6" t="n">
-        <v>516</v>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Public (out-of-state COA)</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>A reasonable hold if you want one large academic medicine option beyond California, but not as safe as the true private/community fits.</t>
-        </is>
-      </c>
-      <c r="L27" s="3" t="inlineStr">
-        <is>
-          <t>The Ohio State University College of Medicine seeks to recruit self-directed learners who are driven to become empathetic physicians providing evidence-based, compassionate medical care.  The Admissions Committee will assemble a class that displays diversity in background and thought, strong intellect, and the potential to improve people's lives through innovation in research, education, patient care and community service.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="32" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Tufts University School of Medicine</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Boston, MA</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>111854</v>
-      </c>
-      <c r="E28" s="5" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="F28" s="6" t="n">
-        <v>516</v>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>Humanistic and community-focused; more realistic than the prestige schools removed, though still not a pure safety.</t>
-        </is>
-      </c>
-      <c r="L28" s="3" t="inlineStr">
-        <is>
-          <t>The mission of Tufts University School of Medicine is to educate a diverse body of students and advance medical knowledge in a dynamic and collaborative environment. We seek to foster the development of dedicated clinicians, scientists, public health professionals, and educators who will have a sustained positive impact on the health of individuals, communities, and the world.
-To achieve the goals of our mission statement, our faculty, students and staff demonstrate our commitment to the following core values in all that we do:
-Commitment to Excellence
-To cultivate a perpetual spirit of inquiry and creativity, leading to outstanding evidence-based health care, rigorous research and scholarship, and inspired teaching.
-Commitment to Humanism
-To relieve suffering and improve quality of life. To treat all people with compassion, respecting human dignity and autonomy.
-Commitment to Social Responsibility
-To serve and advocate for all people, especially underserved and vulnerable patients and populations, by addressing social determinants of health, health equity, social justice, and stewardship of social resources.
-Commitment to Professionalism
-To act in accordance with the highest standards of integrity, demonstrating personal accountability and resilience, collegiality and teamwork, and the pursuit of lifelong learning.
-Tufts University School of Medicine embraces diversity in the broadest form, including racial, ethnic, religious, socioeconomic, geographic diversity, as well as diversity in gender and sexual orientation.
-We believe that inclusive excellence is an essential practice in the creation of a teaching and learning environment that promotes quality, excellence, and equity as core values among our future physicians, scientists and public health advocates; a workforce equipped with the knowledge and skill needed to address the range of health challenges facing our increasingly diverse patient population and their communities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="32" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>University of Illinois College of Medicine</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Chicago, IL</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="n">
-        <v>123095</v>
-      </c>
-      <c r="E29" s="5" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="F29" s="6" t="n">
-        <v>512</v>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Public (out-of-state COA)</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr">
-        <is>
-          <t>Public-school add with some out-of-state risk, but still a useful lower-tier target because its prompts and mission fit you well and the academic bar is manageable.</t>
-        </is>
-      </c>
-      <c r="L29" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">To advance health for everyone through outstanding education, research, clinical care, and social responsibility.
 Mission in Action: We achieve this mission through an innovative and evolving curriculum that integrates the basic, clinical and social sciences, and through a learning environment that emphasizes self-directed, individualized and experiential learning on three 
@@ -2075,117 +1839,57 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>University of Iowa Roy J. and Lucille A. Carver College of Medicine</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Iowa City, IA</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="n">
-        <v>92614</v>
-      </c>
-      <c r="E30" s="5" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="F30" s="6" t="n">
-        <v>516</v>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>University of Massachusetts Chan Medical School</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Worcester, MA</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>113221</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>514</v>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>Public (out-of-state COA)</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>Still competitive, but its out-of-state interview pattern is healthier than many public peers you could have chosen instead.</t>
-        </is>
-      </c>
-      <c r="L30" s="3" t="inlineStr">
-        <is>
-          <t>The Admissions Committee for the University of Iowa Roy J. and Lucille A. Carver College of Medicine admits students who have a genuine interest in the study and practice of medicine; show a desire and commitment to serve the public in matters of health; and who have the personal, professional and intellectual skills and characteristics required to become and competent and caring physician. 
-Personal qualities considered by the Admissions Committee include high moral character, independent thinking, the ability to communicate and interact with others in a sensitive and caring way, the ability to maintain professionalism in stressful situations, and dedication to the idea of service.
-Understanding the importance of the educational benefits resulting from a diverse student population and the interest by the medical profession in serving the healthcare needs of a changing American population, the Admissions Committee values each applicant’s unique strengths, experiences and background.
-To execute our mission, the committee utilizes a holistic review of all candidates. Our committee values each candidates' different experiences and personal stories and takes into consideration: first generation college students, rural backgrounds and experiences, socioeconomic status, and any other impactful experiences students describe in their application that will make them a compassionate and excellent physician.
-Please read our sections about Campus Life to learn more about how Carver's mission informs our culture of collaboration and other initiatives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="32" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>University of Massachusetts Chan Medical School</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Worcester, MA</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="n">
-        <v>113221</v>
-      </c>
-      <c r="E31" s="5" t="n">
-        <v>3.86</v>
-      </c>
-      <c r="F31" s="6" t="n">
-        <v>514</v>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Public (out-of-state COA)</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>Best MSAR-driven addition from the last pass: friendlier accepted and matriculant stats with strong public-service mission.</t>
         </is>
       </c>
-      <c r="L31" s="3" t="inlineStr">
+      <c r="L26" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">The mission of UMass Chan Medical School is to advance the health and well-being of the people of the commonwealth and the world through pioneering advances in education, research and health care delivery. 
 The UMass Chan Medical School Office of Admissions is committed to employing the most effective and evidence-based methods to recruit and matriculate future physicians and scientists who will provide the highest quality medical care for our communities in keeping with the mission of the T.H. Chan School of Medicine.  Our graduates will contribute in a meaningful way to the elimination of health care disparities and the establishment of health equity in Massachusetts and beyond.
@@ -2197,53 +1901,53 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="32" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>University of Wisconsin School of Medicine and Public Health</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="4" t="n">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="4" t="n">
         <v>97464</v>
       </c>
-      <c r="E32" s="5" t="n">
+      <c r="E27" s="5" t="n">
         <v>3.87</v>
       </c>
-      <c r="F32" s="6" t="n">
+      <c r="F27" s="6" t="n">
         <v>512</v>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Public (out-of-state COA)</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>Public-health framing and community mission fit well, though the public-school dynamics keep it out of the safety tier.</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr">
         <is>
           <t>Mission: Together, we are advancing health and health equity through remarkable service to patients and communities, outstanding education, and innovative research.
 Vision: Healthy people. Healthy communities.
@@ -2255,57 +1959,57 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="32" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Vermont Larner College of Medicine</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Burlington, VT</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D28" s="4" t="n">
         <v>105472</v>
       </c>
-      <c r="E33" s="5" t="n">
+      <c r="E28" s="5" t="n">
         <v>3.8</v>
       </c>
-      <c r="F33" s="6" t="n">
+      <c r="F28" s="6" t="n">
         <v>513</v>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>Public (out-of-state COA)</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>Good balance of humanistic training and manageable stats; one of the steadier mission-fit targets on the list.</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">We celebrate over 200 years of excellence in educating physicians and physician-scientists, and in serving our local and global community.
 The mission of the Larner College of Medicine at The University of Vermont is to educate a diverse group of dedicated physicians and biomedical scientists to serve across all the disciplines of medicine; to bring hope to patients by advancing medical knowledge through research; to integrate education and research to advance the quality and accessibility of patient care; and to engage with our communities to benefit Vermont and the world. We achieve this mission through: 
@@ -2321,114 +2025,114 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Wake Forest University School of Medicine</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Winston-Salem, NC</t>
         </is>
       </c>
-      <c r="D34" s="4" t="n">
+      <c r="D29" s="4" t="n">
         <v>110448</v>
       </c>
-      <c r="E34" s="5" t="n">
+      <c r="E29" s="5" t="n">
         <v>3.87</v>
       </c>
-      <c r="F34" s="6" t="n">
+      <c r="F29" s="6" t="n">
         <v>512</v>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>Private</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>Research and service both matter here, making it a more grounded target than the schools removed for prestige-heavy risk.</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">The mission of the Wake Forest University School of Medicine (WFUSM) is to educate future physicians who are empowered to transform health for all. Our vision is to be national leaders in medical education and innovation, graduating purpose-driven physicians committed to improving the health of individuals and communities through lifelong learning.
 </t>
         </is>
       </c>
     </row>
-    <row r="35" ht="32" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Emory University School of Medicine</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Atlanta, GA</t>
         </is>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="D30" s="4" t="n">
         <v>109402</v>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="E30" s="5" t="n">
         <v>3.89</v>
       </c>
-      <c r="F35" s="6" t="n">
+      <c r="F30" s="6" t="n">
         <v>517</v>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>Reach</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>Private</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>Research-forward reach that still rewards service and leadership; worth keeping because your MCAT and conference record help here.</t>
         </is>
       </c>
-      <c r="L35" s="3" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr">
         <is>
           <t>We are committed to recruiting and developing a class of students with the potential to become innovative leaders in biomedical science, public health, medical education, and clinical care. We foster a culture that integrates leading-edge basic, translational, and clinical research to further the ability to deliver quality health care, predict illness, treat the sick, and promote the health of our patients and our communities.  Our mission objectives are as follows:
 -Provide outstanding educational programs for medical and graduate students and healthcare professionals
@@ -2439,177 +2143,286 @@
         </is>
       </c>
     </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Kaiser Permanente Bernard J. Tyson School of Medicine</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Pasadena, CA</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>39636</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>517</v>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Strong humanism-and-equity fit; still selective, but more defensible than some of the private prestige schools that were cut.</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Kaiser Permanente Bernard J. Tyson School of Medicine strives to provide a world-class education for every one of our students.
+We aim to ignite a passion for lifelong learning, a desire to serve patients, and an unwavering commitment to improve the health and well-being of communities.  </t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>New York Medical College</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Valhalla, NY</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>102045</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>517</v>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Private target with room for your high MCAT to help offset GPA risk.</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>New York Medical College is a graduate health sciences university whose purpose is to educate physicians, scientists, public health specialists, and other healthcare professionals, and to conduct biomedical and population-based research. Through its faculty and affiliated clinical partners, the College provides service to its community in an atmosphere of excellence, scholarship, and professionalism. New York Medical College believes the rich diversity of its student body and faculty is important to its mission of educating outstanding health care professionals for the multicultural world of the 21st century. This commitment to diversity and inclusion is woven into the fabric of the institution.  Students come from across the US, representing a broad range of racial, ethnic, cultural, economic, and educational backgrounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>University of California San Diego School of Medicine</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>La Jolla, CA</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>75043</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>516</v>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>CA public (in-state COA)</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Keep as a California reach with strong research upside and a real fit for your research plus service profile.</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>The mission of the UC San Diego School of Medicine is to provide skilled, compassionate physicians well-trained to practice medicine who are sensitive to the needs of the special populations of our region and the nation. In addition, we strive to build on our exceptional biomedical, behavioral and health services research strengths to extend the boundaries of the art and science of medicine through continued research and the preparation of future academicians. In these ways, we also strive to improve the overall health of the population.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>University of Miami Leonard M. Miller School of Medicine</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Miami, FL</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>112815</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>516</v>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>High-upside private reach that still values community-facing work; keep only if you want some ambition in the final list.</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>The University of Miami Miller School of Medicine’s mission is to provide state-of-the-art, translational and evidence-based information to enhance the quality of education, research, and clinical practice, to foster professional growth, to stimulate intellectual (academic) curiosity, and to promote excellence in the delivery of health care in South Florida and internationally. These educational activities will be relevant to medical knowledge, clinical performance, soundly performed research and/or patient outcomes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="3" t="n"/>
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="n"/>
+      <c r="D35" s="4" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="7" t="n"/>
+      <c r="H35" s="3" t="n"/>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+      <c r="L35" s="3" t="n"/>
+    </row>
     <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>Geisel School of Medicine at Dartmouth</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Hanover, NH</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>101004</v>
-      </c>
-      <c r="E36" s="5" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F36" s="6" t="n">
-        <v>517</v>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>Reach</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
-        <is>
-          <t>Still a reach, but the reflective, service-minded, systems-aware fit remains coherent with your essays.</t>
-        </is>
-      </c>
-      <c r="L36" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Our Mission: 
--To improve the lives of the communities we serve through inclusive excellence in learning, discovery, and healing.
--To foster an inclusive, diverse community that reflects our world and addresses the most challenging issues in healthcare.
-At Geisel, our Vision is to be the medical school that sets the standard for educating humanistic physicians, scientists, and educators to be leaders of change and to flourish in their chosen paths . We strive to build a diverse and inclusive community reflective of our world in order to enrich learning, foster innovation, and help tackle the most vexing challenges in health care. We aim to do this by cultivating character, a growth mindset and servant leadership qualities in our students so that they may best serve our communities locally and globally to live healthier and fulfilled lives.
-</t>
-        </is>
-      </c>
+      <c r="A36" s="3" t="n"/>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="7" t="n"/>
+      <c r="H36" s="3" t="n"/>
+      <c r="I36" s="3" t="n"/>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+      <c r="L36" s="3" t="n"/>
     </row>
     <row r="37" ht="32" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>University of California San Diego School of Medicine</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>La Jolla, CA</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>75043</v>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>516</v>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>Reach</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>CA public (in-state COA)</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K37" s="3" t="inlineStr">
-        <is>
-          <t>Keep as a California reach with strong research upside and a real fit for your research plus service profile.</t>
-        </is>
-      </c>
-      <c r="L37" s="3" t="inlineStr">
-        <is>
-          <t>The mission of the UC San Diego School of Medicine is to provide skilled, compassionate physicians well-trained to practice medicine who are sensitive to the needs of the special populations of our region and the nation. In addition, we strive to build on our exceptional biomedical, behavioral and health services research strengths to extend the boundaries of the art and science of medicine through continued research and the preparation of future academicians. In these ways, we also strive to improve the overall health of the population.</t>
-        </is>
-      </c>
+      <c r="A37" s="3" t="n"/>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+      <c r="L37" s="3" t="n"/>
     </row>
     <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>University of Miami Leonard M. Miller School of Medicine</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Miami, FL</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="n">
-        <v>112815</v>
-      </c>
-      <c r="E38" s="5" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F38" s="6" t="n">
-        <v>516</v>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>Reach</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>MSAR cache: data/msar/2027/md_profiles_summary.json</t>
-        </is>
-      </c>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
-          <t>High-upside private reach that still values community-facing work; keep only if you want some ambition in the final list.</t>
-        </is>
-      </c>
-      <c r="L38" s="3" t="inlineStr">
-        <is>
-          <t>The University of Miami Miller School of Medicine’s mission is to provide state-of-the-art, translational and evidence-based information to enhance the quality of education, research, and clinical practice, to foster professional growth, to stimulate intellectual (academic) curiosity, and to promote excellence in the delivery of health care in South Florida and internationally. These educational activities will be relevant to medical knowledge, clinical performance, soundly performed research and/or patient outcomes.</t>
-        </is>
-      </c>
+      <c r="A38" s="3" t="n"/>
+      <c r="B38" s="3" t="n"/>
+      <c r="C38" s="3" t="n"/>
+      <c r="D38" s="4" t="n"/>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="7" t="n"/>
+      <c r="H38" s="3" t="n"/>
+      <c r="I38" s="3" t="n"/>
+      <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
     </row>
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="3" t="n"/>
@@ -2641,12 +2454,8 @@
     <row r="53"/>
     <row r="54"/>
     <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
-  <autoFilter ref="A4:L38"/>
+  <autoFilter ref="A4:L34"/>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
@@ -2673,7 +2482,7 @@
     <row r="1" ht="19" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Expanded school list notes</t>
+          <t>Selection notes</t>
         </is>
       </c>
     </row>
@@ -2687,28 +2496,28 @@
     <row r="3" ht="19" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>This version keeps the list focused on real-fit MD schools rather than padding with region-locked or population-specific options.</t>
+          <t>This version reflects a live 2027 MSAR pass from the signed-in portal on May 30, 2026.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="19" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>I removed Charles Drew and Western Michigan after a closer review of mission fit, accepted-demographic patterns, and secondary prompt screens.</t>
+          <t>Removed: Geisel, Tufts, Ohio State, and Iowa Carver because their live accepted profiles remained too top-heavy for your GPA and odds goal.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Nova Southeastern MD was added as the cleaner lower-tier replacement; I did not force a second replacement because the remaining &lt;=3.85 alternatives were more state- or region-restricted.</t>
+          <t>I kept some mission-coherent reaches, but reclassified schools like Kaiser and NYMC upward in risk to better match the live data.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Current active list size: 34. 'Safety' still means lower relative risk, not a guarantee.</t>
+          <t>Current active list size: 30. 'Safety' still means lower relative risk, not a guarantee.</t>
         </is>
       </c>
     </row>

</xml_diff>